<commit_message>
Some updates soil C pars
</commit_message>
<xml_diff>
--- a/data/default/SoilC-crop_resid.xlsx
+++ b/data/default/SoilC-crop_resid.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jnka0003\Git repos\CIBUSmod\data\default\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B5C3A374-7429-4829-B46D-C34991D5D955}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F72D02D7-DCF8-47DE-948E-76855495D7A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1125" yWindow="1125" windowWidth="21600" windowHeight="12645" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="data" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="168" uniqueCount="122">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="172" uniqueCount="125">
   <si>
     <t>f_crop</t>
   </si>
@@ -228,21 +228,6 @@
     <t>Buckwheat</t>
   </si>
   <si>
-    <t>Bolinder et al 2007: Barley</t>
-  </si>
-  <si>
-    <t>Bolinder et al 2007: Oats</t>
-  </si>
-  <si>
-    <t>Bolinder et al 2007: Small-grain cereals</t>
-  </si>
-  <si>
-    <t>Bolinder et al 2007: Triticale</t>
-  </si>
-  <si>
-    <t>Bolinder et al 2007: Grain-corn</t>
-  </si>
-  <si>
     <t>Jacobs et al 2020: Fodder and vegetable legumes (grains)</t>
   </si>
   <si>
@@ -252,12 +237,6 @@
     <t>Jacobs et al 2020: Oilseed rape</t>
   </si>
   <si>
-    <t>Jacobs et al 2020: Sugar beet</t>
-  </si>
-  <si>
-    <t>Jacobs et al 2020: Potatoes</t>
-  </si>
-  <si>
     <t>Jacobs et al 2020: Clover (seeds)</t>
   </si>
   <si>
@@ -403,6 +382,36 @@
   </si>
   <si>
     <t>Same as Strawberries for now just to have something</t>
+  </si>
+  <si>
+    <t>Net primary productivity and below-ground crop residue inputs for root crops: Potato (Solanum tuberosum L.) and sugar beet (Beta vulgaris L.)</t>
+  </si>
+  <si>
+    <t>https://doi.org/10.4141/cjss-2014-091</t>
+  </si>
+  <si>
+    <t>Bolinder et al (2015)</t>
+  </si>
+  <si>
+    <t>Bolinder et al (2015); R_E=R_R*0.65</t>
+  </si>
+  <si>
+    <t>rhizodep</t>
+  </si>
+  <si>
+    <t>Jacobs et al 2020: Winter barley</t>
+  </si>
+  <si>
+    <t>Jacobs et al 2020: Spring barley</t>
+  </si>
+  <si>
+    <t>Jacobs et al 2020: Oat</t>
+  </si>
+  <si>
+    <t>Jacobs et al 2020: Winter triticale</t>
+  </si>
+  <si>
+    <t>Jacobs et al 2020: Corn, sweet corn</t>
   </si>
 </sst>
 </file>
@@ -413,7 +422,7 @@
     <numFmt numFmtId="164" formatCode="0.000"/>
     <numFmt numFmtId="165" formatCode="0.0"/>
   </numFmts>
-  <fonts count="10" x14ac:knownFonts="1">
+  <fonts count="12" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -491,6 +500,22 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <u/>
+      <sz val="11"/>
+      <color theme="7"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="7"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -519,7 +544,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -571,17 +596,21 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -875,18 +904,18 @@
     <col min="5" max="12" width="9.140625" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>83</v>
+        <v>76</v>
       </c>
       <c r="C1" s="2" t="s">
         <v>1</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>74</v>
+        <v>67</v>
       </c>
       <c r="E1" s="2" t="s">
         <v>2</v>
@@ -914,8 +943,11 @@
       </c>
       <c r="N1" s="2"/>
       <c r="T1" s="12"/>
-    </row>
-    <row r="2" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="X1" s="30" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="2" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>10</v>
       </c>
@@ -951,11 +983,15 @@
         <v>1</v>
       </c>
       <c r="N2" t="s">
-        <v>76</v>
+        <v>69</v>
       </c>
       <c r="T2" s="13"/>
-    </row>
-    <row r="3" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="X2" s="31">
+        <f>H2/G2</f>
+        <v>0.31052631578947365</v>
+      </c>
+    </row>
+    <row r="3" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>11</v>
       </c>
@@ -991,11 +1027,15 @@
         <v>1</v>
       </c>
       <c r="N3" t="s">
-        <v>77</v>
+        <v>70</v>
       </c>
       <c r="T3" s="13"/>
-    </row>
-    <row r="4" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="X3" s="31">
+        <f t="shared" ref="X3:X54" si="0">H3/G3</f>
+        <v>0.31</v>
+      </c>
+    </row>
+    <row r="4" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>12</v>
       </c>
@@ -1031,11 +1071,15 @@
         <v>1</v>
       </c>
       <c r="N4" t="s">
-        <v>78</v>
+        <v>71</v>
       </c>
       <c r="T4" s="13"/>
-    </row>
-    <row r="5" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="X4" s="31">
+        <f t="shared" si="0"/>
+        <v>0.30898876404494385</v>
+      </c>
+    </row>
+    <row r="5" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>13</v>
       </c>
@@ -1046,16 +1090,16 @@
         <v>1</v>
       </c>
       <c r="E5" s="3">
-        <v>0.45100000000000001</v>
+        <v>0.44400000000000001</v>
       </c>
       <c r="F5" s="3">
-        <v>0.4</v>
+        <v>0.32800000000000001</v>
       </c>
       <c r="G5" s="3">
-        <v>0.09</v>
+        <v>0.17399999999999999</v>
       </c>
       <c r="H5" s="3">
-        <v>5.8999999999999997E-2</v>
+        <v>5.3999999999999999E-2</v>
       </c>
       <c r="I5" s="4">
         <v>0</v>
@@ -1070,11 +1114,15 @@
         <v>1</v>
       </c>
       <c r="N5" t="s">
-        <v>63</v>
+        <v>120</v>
       </c>
       <c r="T5" s="13"/>
-    </row>
-    <row r="6" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="X5" s="31">
+        <f t="shared" si="0"/>
+        <v>0.31034482758620691</v>
+      </c>
+    </row>
+    <row r="6" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>14</v>
       </c>
@@ -1085,16 +1133,16 @@
         <v>1</v>
       </c>
       <c r="E6" s="3">
-        <v>0.45100000000000001</v>
+        <v>0.42199999999999999</v>
       </c>
       <c r="F6" s="3">
-        <v>0.4</v>
+        <v>0.315</v>
       </c>
       <c r="G6" s="3">
-        <v>0.09</v>
+        <v>0.2</v>
       </c>
       <c r="H6" s="3">
-        <v>5.8999999999999997E-2</v>
+        <v>6.2E-2</v>
       </c>
       <c r="I6" s="4">
         <v>0</v>
@@ -1109,11 +1157,15 @@
         <v>1</v>
       </c>
       <c r="N6" t="s">
-        <v>63</v>
+        <v>121</v>
       </c>
       <c r="T6" s="13"/>
-    </row>
-    <row r="7" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="X6" s="31">
+        <f t="shared" si="0"/>
+        <v>0.31</v>
+      </c>
+    </row>
+    <row r="7" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>15</v>
       </c>
@@ -1124,16 +1176,16 @@
         <v>1</v>
       </c>
       <c r="E7" s="3">
-        <v>0.31900000000000001</v>
+        <v>0.312</v>
       </c>
       <c r="F7" s="3">
-        <v>0.28299999999999997</v>
+        <v>0.33899999999999997</v>
       </c>
       <c r="G7" s="3">
-        <v>0.24099999999999999</v>
+        <v>0.26700000000000002</v>
       </c>
       <c r="H7" s="3">
-        <v>0.157</v>
+        <v>8.3000000000000004E-2</v>
       </c>
       <c r="I7" s="4">
         <v>0</v>
@@ -1148,11 +1200,15 @@
         <v>1</v>
       </c>
       <c r="N7" t="s">
-        <v>64</v>
+        <v>122</v>
       </c>
       <c r="T7" s="13"/>
-    </row>
-    <row r="8" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="X7" s="31">
+        <f t="shared" si="0"/>
+        <v>0.31086142322097376</v>
+      </c>
+    </row>
+    <row r="8" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>16</v>
       </c>
@@ -1163,16 +1219,16 @@
         <v>1</v>
       </c>
       <c r="E8" s="3">
-        <v>0.26</v>
+        <v>0.42099999999999999</v>
       </c>
       <c r="F8" s="3">
-        <v>0.65600000000000003</v>
+        <v>0.38400000000000001</v>
       </c>
       <c r="G8" s="3">
-        <v>7.4999999999999997E-2</v>
+        <v>0.14899999999999999</v>
       </c>
       <c r="H8" s="3">
-        <v>0.05</v>
+        <v>4.5999999999999999E-2</v>
       </c>
       <c r="I8" s="4">
         <v>0</v>
@@ -1187,11 +1243,15 @@
         <v>1</v>
       </c>
       <c r="N8" t="s">
-        <v>66</v>
+        <v>123</v>
       </c>
       <c r="T8" s="13"/>
-    </row>
-    <row r="9" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="X8" s="31">
+        <f t="shared" si="0"/>
+        <v>0.3087248322147651</v>
+      </c>
+    </row>
+    <row r="9" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>17</v>
       </c>
@@ -1202,16 +1262,16 @@
         <v>1</v>
       </c>
       <c r="E9" s="3">
-        <v>0.26</v>
+        <v>0.42199999999999999</v>
       </c>
       <c r="F9" s="3">
-        <v>0.65600000000000003</v>
+        <v>0.315</v>
       </c>
       <c r="G9" s="3">
-        <v>7.4999999999999997E-2</v>
+        <v>0.2</v>
       </c>
       <c r="H9" s="3">
-        <v>0.05</v>
+        <v>6.2E-2</v>
       </c>
       <c r="I9" s="4">
         <v>0</v>
@@ -1226,11 +1286,15 @@
         <v>1</v>
       </c>
       <c r="N9" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="T9" s="13"/>
-    </row>
-    <row r="10" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="X9" s="31">
+        <f t="shared" si="0"/>
+        <v>0.31</v>
+      </c>
+    </row>
+    <row r="10" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>18</v>
       </c>
@@ -1241,16 +1305,16 @@
         <v>1</v>
       </c>
       <c r="E10" s="3">
-        <v>0.38600000000000001</v>
+        <v>0.39600000000000002</v>
       </c>
       <c r="F10" s="3">
-        <v>0.38700000000000001</v>
+        <v>0.35</v>
       </c>
       <c r="G10" s="3">
-        <v>0.13800000000000001</v>
+        <v>0.19400000000000001</v>
       </c>
       <c r="H10" s="3">
-        <v>8.8999999999999996E-2</v>
+        <v>0.06</v>
       </c>
       <c r="I10" s="4">
         <v>0</v>
@@ -1265,11 +1329,15 @@
         <v>1</v>
       </c>
       <c r="N10" t="s">
-        <v>67</v>
+        <v>124</v>
       </c>
       <c r="T10" s="13"/>
-    </row>
-    <row r="11" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="X10" s="31">
+        <f t="shared" si="0"/>
+        <v>0.30927835051546387</v>
+      </c>
+    </row>
+    <row r="11" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>19</v>
       </c>
@@ -1280,16 +1348,16 @@
         <v>1</v>
       </c>
       <c r="E11" s="3">
-        <v>0.33500000000000002</v>
+        <v>0.42199999999999999</v>
       </c>
       <c r="F11" s="3">
-        <v>0.48199999999999998</v>
+        <v>0.315</v>
       </c>
       <c r="G11" s="3">
-        <v>0.11</v>
+        <v>0.2</v>
       </c>
       <c r="H11" s="3">
-        <v>7.2999999999999995E-2</v>
+        <v>6.2E-2</v>
       </c>
       <c r="I11" s="4">
         <v>0</v>
@@ -1304,11 +1372,15 @@
         <v>1</v>
       </c>
       <c r="N11" t="s">
-        <v>65</v>
+        <v>70</v>
       </c>
       <c r="T11" s="13"/>
-    </row>
-    <row r="12" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="X11" s="31">
+        <f t="shared" si="0"/>
+        <v>0.31</v>
+      </c>
+    </row>
+    <row r="12" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>20</v>
       </c>
@@ -1344,11 +1416,15 @@
         <v>1</v>
       </c>
       <c r="N12" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="T12" s="13"/>
-    </row>
-    <row r="13" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="X12" s="31">
+        <f t="shared" si="0"/>
+        <v>0.31325301204819272</v>
+      </c>
+    </row>
+    <row r="13" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>21</v>
       </c>
@@ -1384,11 +1460,15 @@
         <v>1</v>
       </c>
       <c r="N13" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="T13" s="13"/>
-    </row>
-    <row r="14" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="X13" s="31">
+        <f t="shared" si="0"/>
+        <v>0.31325301204819272</v>
+      </c>
+    </row>
+    <row r="14" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>22</v>
       </c>
@@ -1424,11 +1504,15 @@
         <v>1</v>
       </c>
       <c r="N14" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="T14" s="13"/>
-    </row>
-    <row r="15" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="X14" s="31">
+        <f t="shared" si="0"/>
+        <v>0.31325301204819272</v>
+      </c>
+    </row>
+    <row r="15" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>23</v>
       </c>
@@ -1464,11 +1548,15 @@
         <v>1</v>
       </c>
       <c r="N15" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="T15" s="13"/>
-    </row>
-    <row r="16" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="X15" s="31">
+        <f t="shared" si="0"/>
+        <v>0.31325301204819272</v>
+      </c>
+    </row>
+    <row r="16" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>24</v>
       </c>
@@ -1504,9 +1592,13 @@
         <v>1</v>
       </c>
       <c r="N16" t="s">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="T16" s="13"/>
+      <c r="X16" s="31">
+        <f t="shared" si="0"/>
+        <v>0.31081081081081086</v>
+      </c>
     </row>
     <row r="17" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
@@ -1544,9 +1636,13 @@
         <v>1</v>
       </c>
       <c r="N17" t="s">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="T17" s="13"/>
+      <c r="X17" s="31">
+        <f t="shared" si="0"/>
+        <v>0.31081081081081086</v>
+      </c>
     </row>
     <row r="18" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
@@ -1558,17 +1654,21 @@
       <c r="D18" s="2">
         <v>1</v>
       </c>
-      <c r="E18" s="3">
-        <v>0.79800000000000004</v>
-      </c>
-      <c r="F18" s="3">
-        <v>0.16</v>
-      </c>
-      <c r="G18" s="3">
-        <v>3.3000000000000002E-2</v>
-      </c>
-      <c r="H18" s="3">
-        <v>0.01</v>
+      <c r="E18" s="29">
+        <f>S18/SUM($S18:$V18)</f>
+        <v>0.72718327183271825</v>
+      </c>
+      <c r="F18" s="29">
+        <f>T18/SUM($S18:$V18)</f>
+        <v>0.2322263222632226</v>
+      </c>
+      <c r="G18" s="29">
+        <f>U18/SUM($S18:$V18)</f>
+        <v>2.4600246002460024E-2</v>
+      </c>
+      <c r="H18" s="29">
+        <f>V18/SUM($S18:$V18)</f>
+        <v>1.5990159901599015E-2</v>
       </c>
       <c r="I18" s="4">
         <v>0</v>
@@ -1583,9 +1683,25 @@
         <v>1</v>
       </c>
       <c r="N18" t="s">
-        <v>72</v>
-      </c>
-      <c r="T18" s="13"/>
+        <v>118</v>
+      </c>
+      <c r="S18" s="25">
+        <v>0.73899999999999999</v>
+      </c>
+      <c r="T18" s="28">
+        <v>0.23599999999999999</v>
+      </c>
+      <c r="U18" s="25">
+        <v>2.5000000000000001E-2</v>
+      </c>
+      <c r="V18" s="28">
+        <f>U18*0.65</f>
+        <v>1.6250000000000001E-2</v>
+      </c>
+      <c r="X18" s="31">
+        <f t="shared" si="0"/>
+        <v>0.64999999999999991</v>
+      </c>
     </row>
     <row r="19" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
@@ -1597,17 +1713,21 @@
       <c r="D19" s="2">
         <v>1</v>
       </c>
-      <c r="E19" s="3">
-        <v>0.79800000000000004</v>
-      </c>
-      <c r="F19" s="3">
-        <v>0.16</v>
-      </c>
-      <c r="G19" s="3">
-        <v>3.3000000000000002E-2</v>
-      </c>
-      <c r="H19" s="3">
-        <v>0.01</v>
+      <c r="E19" s="29">
+        <f>S19/SUM($S19:$V19)</f>
+        <v>0.72718327183271825</v>
+      </c>
+      <c r="F19" s="29">
+        <f>T19/SUM($S19:$V19)</f>
+        <v>0.2322263222632226</v>
+      </c>
+      <c r="G19" s="29">
+        <f>U19/SUM($S19:$V19)</f>
+        <v>2.4600246002460024E-2</v>
+      </c>
+      <c r="H19" s="29">
+        <f>V19/SUM($S19:$V19)</f>
+        <v>1.5990159901599015E-2</v>
       </c>
       <c r="I19" s="4">
         <v>0</v>
@@ -1622,9 +1742,25 @@
         <v>1</v>
       </c>
       <c r="N19" t="s">
-        <v>72</v>
-      </c>
-      <c r="T19" s="13"/>
+        <v>118</v>
+      </c>
+      <c r="S19" s="25">
+        <v>0.73899999999999999</v>
+      </c>
+      <c r="T19" s="28">
+        <v>0.23599999999999999</v>
+      </c>
+      <c r="U19" s="25">
+        <v>2.5000000000000001E-2</v>
+      </c>
+      <c r="V19" s="28">
+        <f>U19*0.65</f>
+        <v>1.6250000000000001E-2</v>
+      </c>
+      <c r="X19" s="31">
+        <f t="shared" si="0"/>
+        <v>0.64999999999999991</v>
+      </c>
     </row>
     <row r="20" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
@@ -1636,17 +1772,21 @@
       <c r="D20" s="2">
         <v>1</v>
       </c>
-      <c r="E20" s="3">
-        <v>0.78800000000000003</v>
-      </c>
-      <c r="F20" s="3">
-        <v>0.16900000000000001</v>
-      </c>
-      <c r="G20" s="3">
-        <v>3.3000000000000002E-2</v>
-      </c>
-      <c r="H20" s="3">
-        <v>0.01</v>
+      <c r="E20" s="29">
+        <f>S20/SUM($S20:$V20)</f>
+        <v>0.61915830077642053</v>
+      </c>
+      <c r="F20" s="29">
+        <f>T20/SUM($S20:$V20)</f>
+        <v>0.35309826418080215</v>
+      </c>
+      <c r="G20" s="29">
+        <f>U20/SUM($S20:$V20)</f>
+        <v>1.6814203056228674E-2</v>
+      </c>
+      <c r="H20" s="29">
+        <f>V20/SUM($S20:$V20)</f>
+        <v>1.0929231986548639E-2</v>
       </c>
       <c r="I20" s="4">
         <v>0</v>
@@ -1661,9 +1801,25 @@
         <v>1</v>
       </c>
       <c r="N20" t="s">
-        <v>71</v>
-      </c>
-      <c r="T20" s="13"/>
+        <v>118</v>
+      </c>
+      <c r="S20" s="25">
+        <v>0.626</v>
+      </c>
+      <c r="T20" s="28">
+        <v>0.35699999999999998</v>
+      </c>
+      <c r="U20" s="25">
+        <v>1.7000000000000001E-2</v>
+      </c>
+      <c r="V20" s="28">
+        <f>U20*0.65</f>
+        <v>1.1050000000000001E-2</v>
+      </c>
+      <c r="X20" s="31">
+        <f t="shared" si="0"/>
+        <v>0.65</v>
+      </c>
     </row>
     <row r="21" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
@@ -1701,12 +1857,16 @@
         <v>1</v>
       </c>
       <c r="N21" t="s">
-        <v>73</v>
-      </c>
-      <c r="R21" s="28" t="s">
-        <v>79</v>
+        <v>66</v>
+      </c>
+      <c r="R21" s="26" t="s">
+        <v>72</v>
       </c>
       <c r="T21" s="13"/>
+      <c r="X21" s="31">
+        <f t="shared" si="0"/>
+        <v>0.3100303951367781</v>
+      </c>
     </row>
     <row r="22" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
@@ -1745,12 +1905,16 @@
         <v>1</v>
       </c>
       <c r="N22" t="s">
-        <v>69</v>
+        <v>64</v>
       </c>
       <c r="R22" s="8">
         <v>10</v>
       </c>
       <c r="T22" s="13"/>
+      <c r="X22" s="31">
+        <f t="shared" si="0"/>
+        <v>0.64946236559139781</v>
+      </c>
       <c r="Z22" s="5"/>
     </row>
     <row r="23" spans="1:26" x14ac:dyDescent="0.25">
@@ -1790,12 +1954,16 @@
         <v>1</v>
       </c>
       <c r="N23" t="s">
-        <v>81</v>
+        <v>74</v>
       </c>
       <c r="R23" s="8">
         <v>1</v>
       </c>
       <c r="T23" s="13"/>
+      <c r="X23" s="31">
+        <f t="shared" si="0"/>
+        <v>0.64896755162241881</v>
+      </c>
     </row>
     <row r="24" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
@@ -1812,38 +1980,42 @@
         <v>0.23300000000000001</v>
       </c>
       <c r="F24" s="6">
-        <f t="shared" ref="F24:L24" si="0">F$22</f>
+        <f t="shared" ref="F24:L24" si="1">F$22</f>
         <v>0</v>
       </c>
       <c r="G24" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0.46500000000000002</v>
       </c>
       <c r="H24" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0.30199999999999999</v>
       </c>
       <c r="I24" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0.1</v>
       </c>
       <c r="J24" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="K24" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0.1</v>
       </c>
       <c r="L24" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="N24" s="5" t="s">
-        <v>119</v>
+        <v>112</v>
       </c>
       <c r="R24" s="7"/>
       <c r="T24" s="13"/>
+      <c r="X24" s="31">
+        <f t="shared" si="0"/>
+        <v>0.64946236559139781</v>
+      </c>
     </row>
     <row r="25" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
@@ -1875,19 +2047,23 @@
         <v>1</v>
       </c>
       <c r="K25" s="9">
-        <f t="shared" ref="K25:K31" si="1">1/R25</f>
+        <f t="shared" ref="K25:K31" si="2">1/R25</f>
         <v>1</v>
       </c>
       <c r="L25" s="4">
         <v>1</v>
       </c>
       <c r="N25" t="s">
-        <v>82</v>
+        <v>75</v>
       </c>
       <c r="R25" s="8">
         <v>1</v>
       </c>
       <c r="T25" s="13"/>
+      <c r="X25" s="31">
+        <f t="shared" si="0"/>
+        <v>0.65</v>
+      </c>
     </row>
     <row r="26" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
@@ -1919,19 +2095,23 @@
         <v>1</v>
       </c>
       <c r="K26" s="9">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0.33333333333333331</v>
       </c>
       <c r="L26" s="4">
         <v>1</v>
       </c>
       <c r="N26" t="s">
-        <v>80</v>
+        <v>73</v>
       </c>
       <c r="R26" s="8">
         <v>3</v>
       </c>
       <c r="T26" s="13"/>
+      <c r="X26" s="31">
+        <f t="shared" si="0"/>
+        <v>0.64935064935064934</v>
+      </c>
     </row>
     <row r="27" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
@@ -1963,19 +2143,23 @@
         <v>1</v>
       </c>
       <c r="K27" s="9">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0.2</v>
       </c>
       <c r="L27" s="4">
         <v>1</v>
       </c>
       <c r="N27" t="s">
-        <v>80</v>
+        <v>73</v>
       </c>
       <c r="R27" s="8">
         <v>5</v>
       </c>
       <c r="T27" s="13"/>
+      <c r="X27" s="31">
+        <f t="shared" si="0"/>
+        <v>0.64935064935064934</v>
+      </c>
       <c r="Z27" s="5"/>
     </row>
     <row r="28" spans="1:26" x14ac:dyDescent="0.25">
@@ -2008,19 +2192,23 @@
         <v>1</v>
       </c>
       <c r="K28" s="9">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0.14285714285714285</v>
       </c>
       <c r="L28" s="4">
         <v>1</v>
       </c>
       <c r="N28" t="s">
-        <v>69</v>
+        <v>64</v>
       </c>
       <c r="R28" s="8">
         <v>7</v>
       </c>
       <c r="T28" s="13"/>
+      <c r="X28" s="31">
+        <f t="shared" si="0"/>
+        <v>0.64946236559139781</v>
+      </c>
       <c r="Z28" s="5"/>
     </row>
     <row r="29" spans="1:26" x14ac:dyDescent="0.25">
@@ -2053,19 +2241,23 @@
         <v>1</v>
       </c>
       <c r="K29" s="9">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>1</v>
       </c>
       <c r="L29" s="4">
         <v>1</v>
       </c>
       <c r="N29" t="s">
-        <v>75</v>
+        <v>68</v>
       </c>
       <c r="R29" s="8">
         <v>1</v>
       </c>
       <c r="T29" s="13"/>
+      <c r="X29" s="31">
+        <f t="shared" si="0"/>
+        <v>0.65217391304347816</v>
+      </c>
     </row>
     <row r="30" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
@@ -2097,19 +2289,23 @@
         <v>1</v>
       </c>
       <c r="K30" s="9">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>1</v>
       </c>
       <c r="L30" s="4">
         <v>1</v>
       </c>
       <c r="N30" t="s">
-        <v>75</v>
+        <v>68</v>
       </c>
       <c r="R30" s="8">
         <v>1</v>
       </c>
       <c r="T30" s="13"/>
+      <c r="X30" s="31">
+        <f t="shared" si="0"/>
+        <v>0.65217391304347816</v>
+      </c>
     </row>
     <row r="31" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
@@ -2141,19 +2337,23 @@
         <v>1</v>
       </c>
       <c r="K31" s="9">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>1</v>
       </c>
       <c r="L31" s="4">
         <v>1</v>
       </c>
       <c r="N31" t="s">
-        <v>75</v>
+        <v>68</v>
       </c>
       <c r="R31" s="8">
         <v>1</v>
       </c>
       <c r="T31" s="13"/>
+      <c r="X31" s="31">
+        <f t="shared" si="0"/>
+        <v>0.65217391304347816</v>
+      </c>
     </row>
     <row r="32" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
@@ -2165,16 +2365,16 @@
       <c r="D32" s="2">
         <v>1</v>
       </c>
-      <c r="E32" s="25">
+      <c r="E32" s="3">
         <v>0.78900000000000003</v>
       </c>
-      <c r="F32" s="25">
+      <c r="F32" s="3">
         <v>0.16800000000000001</v>
       </c>
-      <c r="G32" s="25">
+      <c r="G32" s="3">
         <v>3.3000000000000002E-2</v>
       </c>
-      <c r="H32" s="25">
+      <c r="H32" s="3">
         <v>0.01</v>
       </c>
       <c r="I32" s="4">
@@ -2190,11 +2390,15 @@
         <v>1</v>
       </c>
       <c r="N32" t="s">
-        <v>110</v>
+        <v>103</v>
       </c>
       <c r="T32" s="13"/>
-    </row>
-    <row r="33" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="X32" s="31">
+        <f t="shared" si="0"/>
+        <v>0.30303030303030304</v>
+      </c>
+    </row>
+    <row r="33" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>41</v>
       </c>
@@ -2204,16 +2408,16 @@
       <c r="D33" s="2">
         <v>1</v>
       </c>
-      <c r="E33" s="25">
+      <c r="E33" s="3">
         <v>0.84199999999999997</v>
       </c>
-      <c r="F33" s="25">
+      <c r="F33" s="3">
         <v>0.115</v>
       </c>
-      <c r="G33" s="25">
+      <c r="G33" s="3">
         <v>3.3000000000000002E-2</v>
       </c>
-      <c r="H33" s="25">
+      <c r="H33" s="3">
         <v>0.01</v>
       </c>
       <c r="I33" s="4">
@@ -2229,11 +2433,15 @@
         <v>1</v>
       </c>
       <c r="N33" t="s">
-        <v>111</v>
+        <v>104</v>
       </c>
       <c r="T33" s="13"/>
-    </row>
-    <row r="34" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="X33" s="31">
+        <f t="shared" si="0"/>
+        <v>0.30303030303030304</v>
+      </c>
+    </row>
+    <row r="34" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>42</v>
       </c>
@@ -2243,16 +2451,16 @@
       <c r="D34" s="2">
         <v>1</v>
       </c>
-      <c r="E34" s="25">
+      <c r="E34" s="3">
         <v>0.76900000000000002</v>
       </c>
-      <c r="F34" s="25">
+      <c r="F34" s="3">
         <v>0.188</v>
       </c>
-      <c r="G34" s="25">
+      <c r="G34" s="3">
         <v>3.3000000000000002E-2</v>
       </c>
-      <c r="H34" s="25">
+      <c r="H34" s="3">
         <v>0.01</v>
       </c>
       <c r="I34" s="4">
@@ -2268,11 +2476,15 @@
         <v>1</v>
       </c>
       <c r="N34" t="s">
-        <v>112</v>
+        <v>105</v>
       </c>
       <c r="T34" s="13"/>
-    </row>
-    <row r="35" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="X34" s="31">
+        <f t="shared" si="0"/>
+        <v>0.30303030303030304</v>
+      </c>
+    </row>
+    <row r="35" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>43</v>
       </c>
@@ -2282,16 +2494,16 @@
       <c r="D35" s="2">
         <v>1</v>
       </c>
-      <c r="E35" s="25">
+      <c r="E35" s="3">
         <v>0.58499999999999996</v>
       </c>
-      <c r="F35" s="25">
+      <c r="F35" s="3">
         <v>0.111</v>
       </c>
-      <c r="G35" s="25">
+      <c r="G35" s="3">
         <v>0.23200000000000001</v>
       </c>
-      <c r="H35" s="25">
+      <c r="H35" s="3">
         <v>7.1999999999999995E-2</v>
       </c>
       <c r="I35" s="4">
@@ -2307,11 +2519,15 @@
         <v>1</v>
       </c>
       <c r="N35" t="s">
-        <v>113</v>
+        <v>106</v>
       </c>
       <c r="T35" s="13"/>
-    </row>
-    <row r="36" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="X35" s="31">
+        <f t="shared" si="0"/>
+        <v>0.31034482758620685</v>
+      </c>
+    </row>
+    <row r="36" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>44</v>
       </c>
@@ -2321,16 +2537,16 @@
       <c r="D36" s="2">
         <v>1</v>
       </c>
-      <c r="E36" s="25">
-        <v>0.45</v>
-      </c>
-      <c r="F36" s="25">
+      <c r="E36" s="3">
+        <v>0.45</v>
+      </c>
+      <c r="F36" s="3">
         <v>0.246</v>
       </c>
-      <c r="G36" s="25">
+      <c r="G36" s="3">
         <v>0.23200000000000001</v>
       </c>
-      <c r="H36" s="25">
+      <c r="H36" s="3">
         <v>7.1999999999999995E-2</v>
       </c>
       <c r="I36" s="4">
@@ -2346,11 +2562,15 @@
         <v>1</v>
       </c>
       <c r="N36" t="s">
-        <v>114</v>
+        <v>107</v>
       </c>
       <c r="T36" s="13"/>
-    </row>
-    <row r="37" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="X36" s="31">
+        <f t="shared" si="0"/>
+        <v>0.31034482758620685</v>
+      </c>
+    </row>
+    <row r="37" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>45</v>
       </c>
@@ -2360,16 +2580,16 @@
       <c r="D37" s="2">
         <v>1</v>
       </c>
-      <c r="E37" s="25">
+      <c r="E37" s="3">
         <v>0.52200000000000002</v>
       </c>
-      <c r="F37" s="25">
+      <c r="F37" s="3">
         <v>0.17399999999999999</v>
       </c>
-      <c r="G37" s="25">
+      <c r="G37" s="3">
         <v>0.23200000000000001</v>
       </c>
-      <c r="H37" s="25">
+      <c r="H37" s="3">
         <v>7.1999999999999995E-2</v>
       </c>
       <c r="I37" s="4">
@@ -2385,11 +2605,15 @@
         <v>1</v>
       </c>
       <c r="N37" t="s">
-        <v>115</v>
+        <v>108</v>
       </c>
       <c r="T37" s="13"/>
-    </row>
-    <row r="38" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="X37" s="31">
+        <f t="shared" si="0"/>
+        <v>0.31034482758620685</v>
+      </c>
+    </row>
+    <row r="38" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>46</v>
       </c>
@@ -2399,16 +2623,16 @@
       <c r="D38" s="2">
         <v>1</v>
       </c>
-      <c r="E38" s="25">
+      <c r="E38" s="3">
         <v>0.49</v>
       </c>
-      <c r="F38" s="25">
+      <c r="F38" s="3">
         <v>0.20599999999999999</v>
       </c>
-      <c r="G38" s="25">
+      <c r="G38" s="3">
         <v>0.23200000000000001</v>
       </c>
-      <c r="H38" s="25">
+      <c r="H38" s="3">
         <v>7.1999999999999995E-2</v>
       </c>
       <c r="I38" s="4">
@@ -2424,11 +2648,15 @@
         <v>1</v>
       </c>
       <c r="N38" t="s">
-        <v>116</v>
+        <v>109</v>
       </c>
       <c r="T38" s="13"/>
-    </row>
-    <row r="39" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="X38" s="31">
+        <f t="shared" si="0"/>
+        <v>0.31034482758620685</v>
+      </c>
+    </row>
+    <row r="39" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>47</v>
       </c>
@@ -2438,16 +2666,16 @@
       <c r="D39" s="2">
         <v>1</v>
       </c>
-      <c r="E39" s="25">
+      <c r="E39" s="3">
         <v>0.48299999999999998</v>
       </c>
-      <c r="F39" s="25">
+      <c r="F39" s="3">
         <v>0.121</v>
       </c>
-      <c r="G39" s="25">
+      <c r="G39" s="3">
         <v>0.30199999999999999</v>
       </c>
-      <c r="H39" s="25">
+      <c r="H39" s="3">
         <v>9.4E-2</v>
       </c>
       <c r="I39" s="4">
@@ -2463,11 +2691,15 @@
         <v>1</v>
       </c>
       <c r="N39" t="s">
-        <v>117</v>
+        <v>110</v>
       </c>
       <c r="T39" s="13"/>
-    </row>
-    <row r="40" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="X39" s="31">
+        <f t="shared" si="0"/>
+        <v>0.3112582781456954</v>
+      </c>
+    </row>
+    <row r="40" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>48</v>
       </c>
@@ -2477,16 +2709,16 @@
       <c r="D40" s="2">
         <v>1</v>
       </c>
-      <c r="E40" s="25">
-        <v>0.45</v>
-      </c>
-      <c r="F40" s="25">
+      <c r="E40" s="3">
+        <v>0.45</v>
+      </c>
+      <c r="F40" s="3">
         <v>0.246</v>
       </c>
-      <c r="G40" s="25">
+      <c r="G40" s="3">
         <v>0.23200000000000001</v>
       </c>
-      <c r="H40" s="25">
+      <c r="H40" s="3">
         <v>7.1999999999999995E-2</v>
       </c>
       <c r="I40" s="4">
@@ -2502,11 +2734,15 @@
         <v>1</v>
       </c>
       <c r="N40" t="s">
-        <v>114</v>
+        <v>107</v>
       </c>
       <c r="T40" s="13"/>
-    </row>
-    <row r="41" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="X40" s="31">
+        <f t="shared" si="0"/>
+        <v>0.31034482758620685</v>
+      </c>
+    </row>
+    <row r="41" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>49</v>
       </c>
@@ -2516,19 +2752,19 @@
       <c r="D41" s="2">
         <v>1</v>
       </c>
-      <c r="E41" s="25">
+      <c r="E41" s="3">
         <v>0.30199999999999999</v>
       </c>
-      <c r="F41" s="25">
+      <c r="F41" s="3">
         <v>0.30199999999999999</v>
       </c>
-      <c r="G41" s="25">
+      <c r="G41" s="3">
         <v>0.30199999999999999</v>
       </c>
-      <c r="H41" s="25">
+      <c r="H41" s="3">
         <v>9.4E-2</v>
       </c>
-      <c r="I41" s="26">
+      <c r="I41" s="4">
         <v>0</v>
       </c>
       <c r="J41" s="10">
@@ -2539,18 +2775,22 @@
         <f>1/3</f>
         <v>0.33333333333333331</v>
       </c>
-      <c r="L41" s="26">
+      <c r="L41" s="4">
         <v>1</v>
       </c>
       <c r="N41" t="s">
-        <v>118</v>
-      </c>
-      <c r="R41" s="27" t="s">
-        <v>109</v>
+        <v>111</v>
+      </c>
+      <c r="R41" s="25" t="s">
+        <v>102</v>
       </c>
       <c r="T41" s="13"/>
-    </row>
-    <row r="42" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="X41" s="31">
+        <f t="shared" si="0"/>
+        <v>0.3112582781456954</v>
+      </c>
+    </row>
+    <row r="42" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>50</v>
       </c>
@@ -2565,39 +2805,43 @@
         <v>0.30199999999999999</v>
       </c>
       <c r="F42" s="6">
-        <f t="shared" ref="F42:L46" si="2">F$41</f>
+        <f t="shared" ref="F42:L46" si="3">F$41</f>
         <v>0.30199999999999999</v>
       </c>
       <c r="G42" s="6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0.30199999999999999</v>
       </c>
       <c r="H42" s="6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>9.4E-2</v>
       </c>
       <c r="I42" s="6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="J42" s="6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0.33333333333333331</v>
       </c>
       <c r="K42" s="6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0.33333333333333331</v>
       </c>
       <c r="L42" s="6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>1</v>
       </c>
       <c r="N42" s="5" t="s">
-        <v>121</v>
+        <v>114</v>
       </c>
       <c r="T42" s="13"/>
-    </row>
-    <row r="43" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="X42" s="31">
+        <f t="shared" si="0"/>
+        <v>0.3112582781456954</v>
+      </c>
+    </row>
+    <row r="43" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>51</v>
       </c>
@@ -2608,43 +2852,47 @@
         <v>1</v>
       </c>
       <c r="E43" s="6">
-        <f t="shared" ref="E43:E46" si="3">E$41</f>
+        <f t="shared" ref="E43:E46" si="4">E$41</f>
         <v>0.30199999999999999</v>
       </c>
       <c r="F43" s="6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0.30199999999999999</v>
       </c>
       <c r="G43" s="6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0.30199999999999999</v>
       </c>
       <c r="H43" s="6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>9.4E-2</v>
       </c>
       <c r="I43" s="6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="J43" s="6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0.33333333333333331</v>
       </c>
       <c r="K43" s="6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0.33333333333333331</v>
       </c>
       <c r="L43" s="6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>1</v>
       </c>
       <c r="N43" s="5" t="s">
-        <v>121</v>
+        <v>114</v>
       </c>
       <c r="T43" s="13"/>
-    </row>
-    <row r="44" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="X43" s="31">
+        <f t="shared" si="0"/>
+        <v>0.3112582781456954</v>
+      </c>
+    </row>
+    <row r="44" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>52</v>
       </c>
@@ -2655,43 +2903,47 @@
         <v>1</v>
       </c>
       <c r="E44" s="6">
+        <f t="shared" si="4"/>
+        <v>0.30199999999999999</v>
+      </c>
+      <c r="F44" s="6">
         <f t="shared" si="3"/>
         <v>0.30199999999999999</v>
       </c>
-      <c r="F44" s="6">
-        <f t="shared" si="2"/>
+      <c r="G44" s="6">
+        <f t="shared" si="3"/>
         <v>0.30199999999999999</v>
       </c>
-      <c r="G44" s="6">
-        <f t="shared" si="2"/>
-        <v>0.30199999999999999</v>
-      </c>
       <c r="H44" s="6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>9.4E-2</v>
       </c>
       <c r="I44" s="6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="J44" s="6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0.33333333333333331</v>
       </c>
       <c r="K44" s="6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0.33333333333333331</v>
       </c>
       <c r="L44" s="6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>1</v>
       </c>
       <c r="N44" s="5" t="s">
-        <v>121</v>
+        <v>114</v>
       </c>
       <c r="T44" s="13"/>
-    </row>
-    <row r="45" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="X44" s="31">
+        <f t="shared" si="0"/>
+        <v>0.3112582781456954</v>
+      </c>
+    </row>
+    <row r="45" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>53</v>
       </c>
@@ -2702,43 +2954,47 @@
         <v>1</v>
       </c>
       <c r="E45" s="6">
+        <f t="shared" si="4"/>
+        <v>0.30199999999999999</v>
+      </c>
+      <c r="F45" s="6">
         <f t="shared" si="3"/>
         <v>0.30199999999999999</v>
       </c>
-      <c r="F45" s="6">
-        <f t="shared" si="2"/>
+      <c r="G45" s="6">
+        <f t="shared" si="3"/>
         <v>0.30199999999999999</v>
       </c>
-      <c r="G45" s="6">
-        <f t="shared" si="2"/>
-        <v>0.30199999999999999</v>
-      </c>
       <c r="H45" s="6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>9.4E-2</v>
       </c>
       <c r="I45" s="6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="J45" s="6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0.33333333333333331</v>
       </c>
       <c r="K45" s="6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0.33333333333333331</v>
       </c>
       <c r="L45" s="6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>1</v>
       </c>
       <c r="N45" s="5" t="s">
-        <v>121</v>
+        <v>114</v>
       </c>
       <c r="T45" s="13"/>
-    </row>
-    <row r="46" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="X45" s="31">
+        <f t="shared" si="0"/>
+        <v>0.3112582781456954</v>
+      </c>
+    </row>
+    <row r="46" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>54</v>
       </c>
@@ -2749,43 +3005,47 @@
         <v>1</v>
       </c>
       <c r="E46" s="6">
+        <f t="shared" si="4"/>
+        <v>0.30199999999999999</v>
+      </c>
+      <c r="F46" s="6">
         <f t="shared" si="3"/>
         <v>0.30199999999999999</v>
       </c>
-      <c r="F46" s="6">
-        <f t="shared" si="2"/>
+      <c r="G46" s="6">
+        <f t="shared" si="3"/>
         <v>0.30199999999999999</v>
       </c>
-      <c r="G46" s="6">
-        <f t="shared" si="2"/>
-        <v>0.30199999999999999</v>
-      </c>
       <c r="H46" s="6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>9.4E-2</v>
       </c>
       <c r="I46" s="6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="J46" s="6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0.33333333333333331</v>
       </c>
       <c r="K46" s="6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0.33333333333333331</v>
       </c>
       <c r="L46" s="6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>1</v>
       </c>
       <c r="N46" s="5" t="s">
-        <v>121</v>
+        <v>114</v>
       </c>
       <c r="T46" s="13"/>
-    </row>
-    <row r="47" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="X46" s="31">
+        <f t="shared" si="0"/>
+        <v>0.3112582781456954</v>
+      </c>
+    </row>
+    <row r="47" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A47" s="1" t="s">
         <v>55</v>
       </c>
@@ -2822,11 +3082,15 @@
         <v>1</v>
       </c>
       <c r="N47" t="s">
-        <v>77</v>
+        <v>70</v>
       </c>
       <c r="T47" s="13"/>
-    </row>
-    <row r="48" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="X47" s="31">
+        <f t="shared" si="0"/>
+        <v>0.31</v>
+      </c>
+    </row>
+    <row r="48" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A48" s="1" t="s">
         <v>56</v>
       </c>
@@ -2863,11 +3127,15 @@
         <v>1</v>
       </c>
       <c r="N48" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="T48" s="13"/>
-    </row>
-    <row r="49" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="X48" s="31">
+        <f t="shared" si="0"/>
+        <v>0.31325301204819272</v>
+      </c>
+    </row>
+    <row r="49" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A49" s="1" t="s">
         <v>57</v>
       </c>
@@ -2904,11 +3172,15 @@
         <v>1</v>
       </c>
       <c r="N49" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="T49" s="13"/>
-    </row>
-    <row r="50" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="X49" s="31">
+        <f t="shared" si="0"/>
+        <v>0.31325301204819272</v>
+      </c>
+    </row>
+    <row r="50" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A50" s="1" t="s">
         <v>58</v>
       </c>
@@ -2919,16 +3191,16 @@
       <c r="D50" s="2">
         <v>1</v>
       </c>
-      <c r="E50" s="29">
+      <c r="E50" s="27">
         <v>0.26400000000000001</v>
       </c>
-      <c r="F50" s="29">
+      <c r="F50" s="27">
         <v>0.44600000000000001</v>
       </c>
-      <c r="G50" s="29">
+      <c r="G50" s="27">
         <v>0.222</v>
       </c>
-      <c r="H50" s="29">
+      <c r="H50" s="27">
         <v>6.9000000000000006E-2</v>
       </c>
       <c r="I50" s="4">
@@ -2944,11 +3216,15 @@
         <v>1</v>
       </c>
       <c r="N50" t="s">
-        <v>120</v>
+        <v>113</v>
       </c>
       <c r="T50" s="13"/>
-    </row>
-    <row r="51" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="X50" s="31">
+        <f t="shared" si="0"/>
+        <v>0.31081081081081086</v>
+      </c>
+    </row>
+    <row r="51" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A51" s="1" t="s">
         <v>59</v>
       </c>
@@ -2985,11 +3261,15 @@
         <v>1</v>
       </c>
       <c r="N51" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="T51" s="13"/>
-    </row>
-    <row r="52" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="X51" s="31">
+        <f t="shared" si="0"/>
+        <v>0.31325301204819272</v>
+      </c>
+    </row>
+    <row r="52" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A52" s="1" t="s">
         <v>60</v>
       </c>
@@ -3001,43 +3281,47 @@
         <v>1</v>
       </c>
       <c r="E52" s="6">
-        <f t="shared" ref="E52:L53" si="4">E$41</f>
+        <f t="shared" ref="E52:L53" si="5">E$41</f>
         <v>0.30199999999999999</v>
       </c>
       <c r="F52" s="6">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>0.30199999999999999</v>
       </c>
       <c r="G52" s="6">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>0.30199999999999999</v>
       </c>
       <c r="H52" s="6">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>9.4E-2</v>
       </c>
       <c r="I52" s="6">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="J52" s="6">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>0.33333333333333331</v>
       </c>
       <c r="K52" s="6">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>0.33333333333333331</v>
       </c>
       <c r="L52" s="6">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>1</v>
       </c>
       <c r="N52" s="5" t="s">
-        <v>121</v>
+        <v>114</v>
       </c>
       <c r="T52" s="13"/>
-    </row>
-    <row r="53" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="X52" s="31">
+        <f t="shared" si="0"/>
+        <v>0.3112582781456954</v>
+      </c>
+    </row>
+    <row r="53" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A53" s="1" t="s">
         <v>61</v>
       </c>
@@ -3049,43 +3333,47 @@
         <v>1</v>
       </c>
       <c r="E53" s="6">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>0.30199999999999999</v>
       </c>
       <c r="F53" s="6">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>0.30199999999999999</v>
       </c>
       <c r="G53" s="6">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>0.30199999999999999</v>
       </c>
       <c r="H53" s="6">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>9.4E-2</v>
       </c>
       <c r="I53" s="6">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="J53" s="6">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>0.33333333333333331</v>
       </c>
       <c r="K53" s="6">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>0.33333333333333331</v>
       </c>
       <c r="L53" s="6">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>1</v>
       </c>
       <c r="N53" s="5" t="s">
-        <v>121</v>
+        <v>114</v>
       </c>
       <c r="T53" s="13"/>
-    </row>
-    <row r="54" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="X53" s="31">
+        <f t="shared" si="0"/>
+        <v>0.3112582781456954</v>
+      </c>
+    </row>
+    <row r="54" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A54" s="1" t="s">
         <v>62</v>
       </c>
@@ -3122,11 +3410,15 @@
         <v>1</v>
       </c>
       <c r="N54" t="s">
-        <v>77</v>
+        <v>70</v>
       </c>
       <c r="T54" s="13"/>
-    </row>
-    <row r="55" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="X54" s="31">
+        <f t="shared" si="0"/>
+        <v>0.31</v>
+      </c>
+    </row>
+    <row r="55" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A55" s="1"/>
       <c r="B55" s="1"/>
       <c r="E55" s="6"/>
@@ -3139,9 +3431,9 @@
       <c r="L55" s="4"/>
       <c r="T55" s="13"/>
     </row>
-    <row r="56" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A56" s="17" t="s">
-        <v>104</v>
+        <v>97</v>
       </c>
       <c r="B56" s="18"/>
       <c r="C56" s="19"/>
@@ -3164,37 +3456,37 @@
       <c r="T56" s="23"/>
       <c r="U56" s="22"/>
     </row>
-    <row r="57" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:24" x14ac:dyDescent="0.25">
       <c r="I57" s="4"/>
       <c r="J57" s="4"/>
       <c r="K57" s="4"/>
       <c r="L57" s="4"/>
       <c r="N57" s="14" t="s">
-        <v>85</v>
+        <v>78</v>
       </c>
       <c r="T57" s="13"/>
     </row>
-    <row r="58" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
         <v>10</v>
       </c>
       <c r="B58" t="s">
-        <v>84</v>
+        <v>77</v>
       </c>
       <c r="E58" s="3">
-        <f t="shared" ref="E58:F67" si="5">E2 / SUM($E2,$F2,$G2*$N58,$H2*$N58)</f>
+        <f t="shared" ref="E58:F67" si="6">E2 / SUM($E2,$F2,$G2*$N58,$H2*$N58)</f>
         <v>0.37083148065807031</v>
       </c>
       <c r="F58" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>0.29702089817696753</v>
       </c>
       <c r="G58" s="3">
-        <f t="shared" ref="G58:H67" si="6">G2*$N58 / SUM($E2,$F2,$G2*$N58,$H2*$N58)</f>
+        <f t="shared" ref="G58:H67" si="7">G2*$N58 / SUM($E2,$F2,$G2*$N58,$H2*$N58)</f>
         <v>0.25344597598932861</v>
       </c>
       <c r="H58" s="3">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>7.8701645175633606E-2</v>
       </c>
       <c r="N58" s="2">
@@ -3202,178 +3494,178 @@
         <v>1.4999999999999998</v>
       </c>
       <c r="P58" t="s">
-        <v>103</v>
+        <v>96</v>
       </c>
       <c r="T58" s="13"/>
     </row>
-    <row r="59" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>11</v>
       </c>
       <c r="B59" t="s">
-        <v>84</v>
+        <v>77</v>
       </c>
       <c r="E59" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>0.37345132743362836</v>
       </c>
       <c r="F59" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>0.2787610619469027</v>
       </c>
       <c r="G59" s="3">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>0.26548672566371689</v>
       </c>
       <c r="H59" s="3">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>8.2300884955752218E-2</v>
       </c>
       <c r="N59" s="2">
         <v>1.5</v>
       </c>
       <c r="P59" s="16" t="s">
-        <v>102</v>
+        <v>95</v>
       </c>
       <c r="T59" s="13"/>
     </row>
-    <row r="60" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>12</v>
       </c>
       <c r="B60" t="s">
-        <v>84</v>
+        <v>77</v>
       </c>
       <c r="E60" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>0.3621694307485433</v>
       </c>
       <c r="F60" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>0.3245181532944868</v>
       </c>
       <c r="G60" s="3">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>0.23935454952935906</v>
       </c>
       <c r="H60" s="3">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>7.3957866427610944E-2</v>
       </c>
       <c r="N60" s="2">
         <v>1.5</v>
       </c>
       <c r="P60" s="16" t="s">
-        <v>107</v>
+        <v>100</v>
       </c>
       <c r="T60" s="13"/>
     </row>
-    <row r="61" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
         <v>13</v>
       </c>
       <c r="B61" t="s">
-        <v>84</v>
+        <v>77</v>
       </c>
       <c r="E61" s="3">
-        <f t="shared" si="5"/>
-        <v>0.41973010702652397</v>
+        <f t="shared" si="6"/>
+        <v>0.39856373429084385</v>
       </c>
       <c r="F61" s="3">
-        <f t="shared" si="5"/>
-        <v>0.37226617031177295</v>
+        <f t="shared" si="6"/>
+        <v>0.29443447037701981</v>
       </c>
       <c r="G61" s="3">
-        <f t="shared" si="6"/>
-        <v>0.12563983248022337</v>
+        <f t="shared" si="7"/>
+        <v>0.23429084380610415</v>
       </c>
       <c r="H61" s="3">
-        <f t="shared" si="6"/>
-        <v>8.2363890181479757E-2</v>
+        <f t="shared" si="7"/>
+        <v>7.2710951526032325E-2</v>
       </c>
       <c r="N61" s="2">
         <v>1.5</v>
       </c>
       <c r="T61" s="13"/>
     </row>
-    <row r="62" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>14</v>
       </c>
       <c r="B62" t="s">
-        <v>84</v>
+        <v>77</v>
       </c>
       <c r="E62" s="3">
-        <f t="shared" si="5"/>
-        <v>0.41973010702652397</v>
+        <f t="shared" si="6"/>
+        <v>0.37345132743362836</v>
       </c>
       <c r="F62" s="3">
-        <f t="shared" si="5"/>
-        <v>0.37226617031177295</v>
+        <f t="shared" si="6"/>
+        <v>0.2787610619469027</v>
       </c>
       <c r="G62" s="3">
-        <f t="shared" si="6"/>
-        <v>0.12563983248022337</v>
+        <f t="shared" si="7"/>
+        <v>0.26548672566371689</v>
       </c>
       <c r="H62" s="3">
-        <f t="shared" si="6"/>
-        <v>8.2363890181479757E-2</v>
+        <f t="shared" si="7"/>
+        <v>8.2300884955752218E-2</v>
       </c>
       <c r="N62" s="2">
         <v>1.5</v>
       </c>
       <c r="T62" s="13"/>
     </row>
-    <row r="63" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
         <v>15</v>
       </c>
       <c r="B63" t="s">
-        <v>84</v>
+        <v>77</v>
       </c>
       <c r="E63" s="3">
-        <f t="shared" si="5"/>
-        <v>0.26605504587155965</v>
+        <f t="shared" si="6"/>
+        <v>0.26530612244897955</v>
       </c>
       <c r="F63" s="3">
-        <f t="shared" si="5"/>
-        <v>0.23603002502085069</v>
+        <f t="shared" si="6"/>
+        <v>0.28826530612244894</v>
       </c>
       <c r="G63" s="3">
-        <f t="shared" si="6"/>
-        <v>0.30150125104253545</v>
+        <f t="shared" si="7"/>
+        <v>0.34056122448979587</v>
       </c>
       <c r="H63" s="3">
-        <f t="shared" si="6"/>
-        <v>0.19641367806505419</v>
+        <f t="shared" si="7"/>
+        <v>0.10586734693877549</v>
       </c>
       <c r="N63" s="2">
         <v>1.5</v>
       </c>
       <c r="T63" s="13"/>
     </row>
-    <row r="64" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
         <v>16</v>
       </c>
       <c r="B64" t="s">
-        <v>84</v>
+        <v>77</v>
       </c>
       <c r="E64" s="3">
-        <f t="shared" si="5"/>
-        <v>0.23561395559583148</v>
+        <f t="shared" si="6"/>
+        <v>0.38359908883826882</v>
       </c>
       <c r="F64" s="3">
-        <f t="shared" si="5"/>
-        <v>0.59447213411871325</v>
+        <f t="shared" si="6"/>
+        <v>0.34988610478359911</v>
       </c>
       <c r="G64" s="3">
-        <f t="shared" si="6"/>
-        <v>0.10194834617127321</v>
+        <f t="shared" si="7"/>
+        <v>0.20364464692482914</v>
       </c>
       <c r="H64" s="3">
-        <f t="shared" si="6"/>
-        <v>6.7965564114182156E-2</v>
+        <f t="shared" si="7"/>
+        <v>6.2870159453302973E-2</v>
       </c>
       <c r="N64" s="2">
         <v>1.5</v>
@@ -3385,23 +3677,23 @@
         <v>17</v>
       </c>
       <c r="B65" t="s">
-        <v>84</v>
+        <v>77</v>
       </c>
       <c r="E65" s="3">
-        <f t="shared" si="5"/>
-        <v>0.23561395559583148</v>
+        <f t="shared" si="6"/>
+        <v>0.37345132743362836</v>
       </c>
       <c r="F65" s="3">
-        <f t="shared" si="5"/>
-        <v>0.59447213411871325</v>
+        <f t="shared" si="6"/>
+        <v>0.2787610619469027</v>
       </c>
       <c r="G65" s="3">
-        <f t="shared" si="6"/>
-        <v>0.10194834617127321</v>
+        <f t="shared" si="7"/>
+        <v>0.26548672566371689</v>
       </c>
       <c r="H65" s="3">
-        <f t="shared" si="6"/>
-        <v>6.7965564114182156E-2</v>
+        <f t="shared" si="7"/>
+        <v>8.2300884955752218E-2</v>
       </c>
       <c r="N65" s="2">
         <v>1.5</v>
@@ -3413,23 +3705,23 @@
         <v>18</v>
       </c>
       <c r="B66" t="s">
-        <v>84</v>
+        <v>77</v>
       </c>
       <c r="E66" s="3">
-        <f t="shared" si="5"/>
-        <v>0.34665469241131569</v>
+        <f t="shared" si="6"/>
+        <v>0.35137533274179239</v>
       </c>
       <c r="F66" s="3">
-        <f t="shared" si="5"/>
-        <v>0.34755276156264037</v>
+        <f t="shared" si="6"/>
+        <v>0.3105590062111801</v>
       </c>
       <c r="G66" s="3">
-        <f t="shared" si="6"/>
-        <v>0.18590031432420298</v>
+        <f t="shared" si="7"/>
+        <v>0.25820763087843834</v>
       </c>
       <c r="H66" s="3">
-        <f t="shared" si="6"/>
-        <v>0.11989223170184106</v>
+        <f t="shared" si="7"/>
+        <v>7.9858030168589167E-2</v>
       </c>
       <c r="N66" s="2">
         <v>1.5</v>
@@ -3441,23 +3733,23 @@
         <v>19</v>
       </c>
       <c r="B67" t="s">
-        <v>84</v>
+        <v>77</v>
       </c>
       <c r="E67" s="3">
-        <f t="shared" si="5"/>
-        <v>0.30691708657810357</v>
+        <f t="shared" si="6"/>
+        <v>0.37345132743362836</v>
       </c>
       <c r="F67" s="3">
-        <f t="shared" si="5"/>
-        <v>0.44159413650939078</v>
+        <f t="shared" si="6"/>
+        <v>0.2787610619469027</v>
       </c>
       <c r="G67" s="3">
-        <f t="shared" si="6"/>
-        <v>0.15116811726981219</v>
+        <f t="shared" si="7"/>
+        <v>0.26548672566371689</v>
       </c>
       <c r="H67" s="3">
-        <f t="shared" si="6"/>
-        <v>0.10032065964269353</v>
+        <f t="shared" si="7"/>
+        <v>8.2300884955752218E-2</v>
       </c>
       <c r="N67" s="2">
         <v>1.5</v>
@@ -3477,7 +3769,7 @@
         <v>34</v>
       </c>
       <c r="B69" t="s">
-        <v>84</v>
+        <v>77</v>
       </c>
       <c r="E69" s="3">
         <f>E26 / SUM($E26,$F26,$G26*$N69,$H26*$N69)</f>
@@ -3500,7 +3792,7 @@
         <v>1.3103448275862069</v>
       </c>
       <c r="P69" t="s">
-        <v>101</v>
+        <v>94</v>
       </c>
       <c r="T69" s="13"/>
     </row>
@@ -3509,7 +3801,7 @@
         <v>35</v>
       </c>
       <c r="B70" t="s">
-        <v>84</v>
+        <v>77</v>
       </c>
       <c r="E70" s="3">
         <f>E27 / SUM($E27,$F27,$G27*$N70,$H27*$N70)</f>
@@ -3532,7 +3824,7 @@
         <v>1.3103448275862069</v>
       </c>
       <c r="P70" s="16" t="s">
-        <v>105</v>
+        <v>98</v>
       </c>
       <c r="T70" s="13"/>
     </row>
@@ -3542,7 +3834,7 @@
       <c r="G71" s="3"/>
       <c r="H71" s="3"/>
       <c r="P71" s="16" t="s">
-        <v>108</v>
+        <v>101</v>
       </c>
     </row>
     <row r="72" spans="1:20" x14ac:dyDescent="0.25">
@@ -3551,7 +3843,7 @@
       <c r="G72" s="3"/>
       <c r="H72" s="3"/>
       <c r="P72" s="16" t="s">
-        <v>106</v>
+        <v>99</v>
       </c>
     </row>
     <row r="73" spans="1:20" x14ac:dyDescent="0.25">
@@ -3639,7 +3931,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ACE673D0-B486-42BC-A4BF-F243D149D98D}">
-  <dimension ref="A1:C5"/>
+  <dimension ref="A1:C6"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="33.85546875" customWidth="1"/>
@@ -3649,57 +3941,68 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="11" t="s">
-        <v>88</v>
+        <v>81</v>
       </c>
       <c r="B1" s="11" t="s">
-        <v>86</v>
+        <v>79</v>
       </c>
       <c r="C1" s="11" t="s">
-        <v>87</v>
+        <v>80</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>91</v>
+        <v>84</v>
       </c>
       <c r="B2" t="s">
-        <v>89</v>
+        <v>82</v>
       </c>
       <c r="C2" s="15" t="s">
-        <v>90</v>
+        <v>83</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>93</v>
+        <v>86</v>
       </c>
       <c r="B3" t="s">
-        <v>94</v>
+        <v>87</v>
       </c>
       <c r="C3" s="15" t="s">
-        <v>92</v>
+        <v>85</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>97</v>
+        <v>90</v>
       </c>
       <c r="B4" t="s">
-        <v>95</v>
+        <v>88</v>
       </c>
       <c r="C4" s="15" t="s">
-        <v>96</v>
+        <v>89</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>98</v>
+        <v>91</v>
       </c>
       <c r="B5" t="s">
-        <v>99</v>
+        <v>92</v>
       </c>
       <c r="C5" s="15" t="s">
-        <v>100</v>
+        <v>93</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>117</v>
+      </c>
+      <c r="B6" t="s">
+        <v>115</v>
+      </c>
+      <c r="C6" s="15" t="s">
+        <v>116</v>
       </c>
     </row>
   </sheetData>
@@ -3708,6 +4011,7 @@
     <hyperlink ref="C3" r:id="rId2" xr:uid="{0EA7DA71-4310-4F21-8C03-6BB56C175491}"/>
     <hyperlink ref="C4" r:id="rId3" xr:uid="{47B930F4-765A-4E76-AE11-48B9DAEFFCE4}"/>
     <hyperlink ref="C5" r:id="rId4" xr:uid="{8F5E3C95-76D5-466C-96CD-FD87EC47CB32}"/>
+    <hyperlink ref="C6" r:id="rId5" xr:uid="{7A81234E-B461-44B2-B0A3-2797A159E6E5}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Implemented more detailed re-values from Bolinder and revised some other SoilC data
</commit_message>
<xml_diff>
--- a/data/default/SoilC-crop_resid.xlsx
+++ b/data/default/SoilC-crop_resid.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jnka0003\Git repos\CIBUSmod\data\default\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F72D02D7-DCF8-47DE-948E-76855495D7A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4742B5F9-86CF-4B1F-87DF-F3428393CDE6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="1725" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="data" sheetId="1" r:id="rId1"/>
@@ -1655,19 +1655,19 @@
         <v>1</v>
       </c>
       <c r="E18" s="29">
-        <f>S18/SUM($S18:$V18)</f>
+        <f t="shared" ref="E18:H20" si="1">S18/SUM($S18:$V18)</f>
         <v>0.72718327183271825</v>
       </c>
       <c r="F18" s="29">
-        <f>T18/SUM($S18:$V18)</f>
+        <f t="shared" si="1"/>
         <v>0.2322263222632226</v>
       </c>
       <c r="G18" s="29">
-        <f>U18/SUM($S18:$V18)</f>
+        <f t="shared" si="1"/>
         <v>2.4600246002460024E-2</v>
       </c>
       <c r="H18" s="29">
-        <f>V18/SUM($S18:$V18)</f>
+        <f t="shared" si="1"/>
         <v>1.5990159901599015E-2</v>
       </c>
       <c r="I18" s="4">
@@ -1714,19 +1714,19 @@
         <v>1</v>
       </c>
       <c r="E19" s="29">
-        <f>S19/SUM($S19:$V19)</f>
+        <f t="shared" si="1"/>
         <v>0.72718327183271825</v>
       </c>
       <c r="F19" s="29">
-        <f>T19/SUM($S19:$V19)</f>
+        <f t="shared" si="1"/>
         <v>0.2322263222632226</v>
       </c>
       <c r="G19" s="29">
-        <f>U19/SUM($S19:$V19)</f>
+        <f t="shared" si="1"/>
         <v>2.4600246002460024E-2</v>
       </c>
       <c r="H19" s="29">
-        <f>V19/SUM($S19:$V19)</f>
+        <f t="shared" si="1"/>
         <v>1.5990159901599015E-2</v>
       </c>
       <c r="I19" s="4">
@@ -1773,19 +1773,19 @@
         <v>1</v>
       </c>
       <c r="E20" s="29">
-        <f>S20/SUM($S20:$V20)</f>
+        <f t="shared" si="1"/>
         <v>0.61915830077642053</v>
       </c>
       <c r="F20" s="29">
-        <f>T20/SUM($S20:$V20)</f>
+        <f t="shared" si="1"/>
         <v>0.35309826418080215</v>
       </c>
       <c r="G20" s="29">
-        <f>U20/SUM($S20:$V20)</f>
+        <f t="shared" si="1"/>
         <v>1.6814203056228674E-2</v>
       </c>
       <c r="H20" s="29">
-        <f>V20/SUM($S20:$V20)</f>
+        <f t="shared" si="1"/>
         <v>1.0929231986548639E-2</v>
       </c>
       <c r="I20" s="4">
@@ -1980,31 +1980,31 @@
         <v>0.23300000000000001</v>
       </c>
       <c r="F24" s="6">
-        <f t="shared" ref="F24:L24" si="1">F$22</f>
+        <f t="shared" ref="F24:L24" si="2">F$22</f>
         <v>0</v>
       </c>
       <c r="G24" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0.46500000000000002</v>
       </c>
       <c r="H24" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0.30199999999999999</v>
       </c>
       <c r="I24" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0.1</v>
       </c>
       <c r="J24" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>1</v>
       </c>
       <c r="K24" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0.1</v>
       </c>
       <c r="L24" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>1</v>
       </c>
       <c r="N24" s="5" t="s">
@@ -2047,7 +2047,7 @@
         <v>1</v>
       </c>
       <c r="K25" s="9">
-        <f t="shared" ref="K25:K31" si="2">1/R25</f>
+        <f t="shared" ref="K25:K31" si="3">1/R25</f>
         <v>1</v>
       </c>
       <c r="L25" s="4">
@@ -2089,14 +2089,14 @@
       </c>
       <c r="I26" s="9">
         <f>0.15*(1/R26)</f>
-        <v>4.9999999999999996E-2</v>
+        <v>0.03</v>
       </c>
       <c r="J26" s="10">
         <v>1</v>
       </c>
       <c r="K26" s="9">
-        <f t="shared" si="2"/>
-        <v>0.33333333333333331</v>
+        <f t="shared" si="3"/>
+        <v>0.2</v>
       </c>
       <c r="L26" s="4">
         <v>1</v>
@@ -2105,7 +2105,7 @@
         <v>73</v>
       </c>
       <c r="R26" s="8">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="T26" s="13"/>
       <c r="X26" s="31">
@@ -2137,14 +2137,14 @@
       </c>
       <c r="I27" s="9">
         <f>(1-0.625)*(1/R27)</f>
-        <v>7.5000000000000011E-2</v>
+        <v>5.3571428571428568E-2</v>
       </c>
       <c r="J27" s="10">
         <v>1</v>
       </c>
       <c r="K27" s="9">
-        <f t="shared" si="2"/>
-        <v>0.2</v>
+        <f t="shared" si="3"/>
+        <v>0.14285714285714285</v>
       </c>
       <c r="L27" s="4">
         <v>1</v>
@@ -2153,7 +2153,7 @@
         <v>73</v>
       </c>
       <c r="R27" s="8">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="T27" s="13"/>
       <c r="X27" s="31">
@@ -2192,7 +2192,7 @@
         <v>1</v>
       </c>
       <c r="K28" s="9">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0.14285714285714285</v>
       </c>
       <c r="L28" s="4">
@@ -2241,7 +2241,7 @@
         <v>1</v>
       </c>
       <c r="K29" s="9">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>1</v>
       </c>
       <c r="L29" s="4">
@@ -2289,7 +2289,7 @@
         <v>1</v>
       </c>
       <c r="K30" s="9">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>1</v>
       </c>
       <c r="L30" s="4">
@@ -2337,7 +2337,7 @@
         <v>1</v>
       </c>
       <c r="K31" s="9">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>1</v>
       </c>
       <c r="L31" s="4">
@@ -2805,31 +2805,31 @@
         <v>0.30199999999999999</v>
       </c>
       <c r="F42" s="6">
-        <f t="shared" ref="F42:L46" si="3">F$41</f>
+        <f t="shared" ref="F42:L46" si="4">F$41</f>
         <v>0.30199999999999999</v>
       </c>
       <c r="G42" s="6">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>0.30199999999999999</v>
       </c>
       <c r="H42" s="6">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>9.4E-2</v>
       </c>
       <c r="I42" s="6">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="J42" s="6">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>0.33333333333333331</v>
       </c>
       <c r="K42" s="6">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>0.33333333333333331</v>
       </c>
       <c r="L42" s="6">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>1</v>
       </c>
       <c r="N42" s="5" t="s">
@@ -2852,35 +2852,35 @@
         <v>1</v>
       </c>
       <c r="E43" s="6">
-        <f t="shared" ref="E43:E46" si="4">E$41</f>
+        <f t="shared" ref="E43:E46" si="5">E$41</f>
         <v>0.30199999999999999</v>
       </c>
       <c r="F43" s="6">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>0.30199999999999999</v>
       </c>
       <c r="G43" s="6">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>0.30199999999999999</v>
       </c>
       <c r="H43" s="6">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>9.4E-2</v>
       </c>
       <c r="I43" s="6">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="J43" s="6">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>0.33333333333333331</v>
       </c>
       <c r="K43" s="6">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>0.33333333333333331</v>
       </c>
       <c r="L43" s="6">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>1</v>
       </c>
       <c r="N43" s="5" t="s">
@@ -2903,35 +2903,35 @@
         <v>1</v>
       </c>
       <c r="E44" s="6">
+        <f t="shared" si="5"/>
+        <v>0.30199999999999999</v>
+      </c>
+      <c r="F44" s="6">
         <f t="shared" si="4"/>
         <v>0.30199999999999999</v>
       </c>
-      <c r="F44" s="6">
-        <f t="shared" si="3"/>
+      <c r="G44" s="6">
+        <f t="shared" si="4"/>
         <v>0.30199999999999999</v>
       </c>
-      <c r="G44" s="6">
-        <f t="shared" si="3"/>
-        <v>0.30199999999999999</v>
-      </c>
       <c r="H44" s="6">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>9.4E-2</v>
       </c>
       <c r="I44" s="6">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="J44" s="6">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>0.33333333333333331</v>
       </c>
       <c r="K44" s="6">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>0.33333333333333331</v>
       </c>
       <c r="L44" s="6">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>1</v>
       </c>
       <c r="N44" s="5" t="s">
@@ -2954,35 +2954,35 @@
         <v>1</v>
       </c>
       <c r="E45" s="6">
+        <f t="shared" si="5"/>
+        <v>0.30199999999999999</v>
+      </c>
+      <c r="F45" s="6">
         <f t="shared" si="4"/>
         <v>0.30199999999999999</v>
       </c>
-      <c r="F45" s="6">
-        <f t="shared" si="3"/>
+      <c r="G45" s="6">
+        <f t="shared" si="4"/>
         <v>0.30199999999999999</v>
       </c>
-      <c r="G45" s="6">
-        <f t="shared" si="3"/>
-        <v>0.30199999999999999</v>
-      </c>
       <c r="H45" s="6">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>9.4E-2</v>
       </c>
       <c r="I45" s="6">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="J45" s="6">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>0.33333333333333331</v>
       </c>
       <c r="K45" s="6">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>0.33333333333333331</v>
       </c>
       <c r="L45" s="6">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>1</v>
       </c>
       <c r="N45" s="5" t="s">
@@ -3005,35 +3005,35 @@
         <v>1</v>
       </c>
       <c r="E46" s="6">
+        <f t="shared" si="5"/>
+        <v>0.30199999999999999</v>
+      </c>
+      <c r="F46" s="6">
         <f t="shared" si="4"/>
         <v>0.30199999999999999</v>
       </c>
-      <c r="F46" s="6">
-        <f t="shared" si="3"/>
+      <c r="G46" s="6">
+        <f t="shared" si="4"/>
         <v>0.30199999999999999</v>
       </c>
-      <c r="G46" s="6">
-        <f t="shared" si="3"/>
-        <v>0.30199999999999999</v>
-      </c>
       <c r="H46" s="6">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>9.4E-2</v>
       </c>
       <c r="I46" s="6">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="J46" s="6">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>0.33333333333333331</v>
       </c>
       <c r="K46" s="6">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>0.33333333333333331</v>
       </c>
       <c r="L46" s="6">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>1</v>
       </c>
       <c r="N46" s="5" t="s">
@@ -3281,35 +3281,35 @@
         <v>1</v>
       </c>
       <c r="E52" s="6">
-        <f t="shared" ref="E52:L53" si="5">E$41</f>
+        <f t="shared" ref="E52:L53" si="6">E$41</f>
         <v>0.30199999999999999</v>
       </c>
       <c r="F52" s="6">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>0.30199999999999999</v>
       </c>
       <c r="G52" s="6">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>0.30199999999999999</v>
       </c>
       <c r="H52" s="6">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>9.4E-2</v>
       </c>
       <c r="I52" s="6">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
       <c r="J52" s="6">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>0.33333333333333331</v>
       </c>
       <c r="K52" s="6">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>0.33333333333333331</v>
       </c>
       <c r="L52" s="6">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>1</v>
       </c>
       <c r="N52" s="5" t="s">
@@ -3333,35 +3333,35 @@
         <v>1</v>
       </c>
       <c r="E53" s="6">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>0.30199999999999999</v>
       </c>
       <c r="F53" s="6">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>0.30199999999999999</v>
       </c>
       <c r="G53" s="6">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>0.30199999999999999</v>
       </c>
       <c r="H53" s="6">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>9.4E-2</v>
       </c>
       <c r="I53" s="6">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
       <c r="J53" s="6">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>0.33333333333333331</v>
       </c>
       <c r="K53" s="6">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>0.33333333333333331</v>
       </c>
       <c r="L53" s="6">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>1</v>
       </c>
       <c r="N53" s="5" t="s">
@@ -3474,19 +3474,19 @@
         <v>77</v>
       </c>
       <c r="E58" s="3">
-        <f t="shared" ref="E58:F67" si="6">E2 / SUM($E2,$F2,$G2*$N58,$H2*$N58)</f>
+        <f t="shared" ref="E58:F67" si="7">E2 / SUM($E2,$F2,$G2*$N58,$H2*$N58)</f>
         <v>0.37083148065807031</v>
       </c>
       <c r="F58" s="3">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>0.29702089817696753</v>
       </c>
       <c r="G58" s="3">
-        <f t="shared" ref="G58:H67" si="7">G2*$N58 / SUM($E2,$F2,$G2*$N58,$H2*$N58)</f>
+        <f t="shared" ref="G58:H67" si="8">G2*$N58 / SUM($E2,$F2,$G2*$N58,$H2*$N58)</f>
         <v>0.25344597598932861</v>
       </c>
       <c r="H58" s="3">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>7.8701645175633606E-2</v>
       </c>
       <c r="N58" s="2">
@@ -3506,19 +3506,19 @@
         <v>77</v>
       </c>
       <c r="E59" s="3">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>0.37345132743362836</v>
       </c>
       <c r="F59" s="3">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>0.2787610619469027</v>
       </c>
       <c r="G59" s="3">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>0.26548672566371689</v>
       </c>
       <c r="H59" s="3">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>8.2300884955752218E-2</v>
       </c>
       <c r="N59" s="2">
@@ -3537,19 +3537,19 @@
         <v>77</v>
       </c>
       <c r="E60" s="3">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>0.3621694307485433</v>
       </c>
       <c r="F60" s="3">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>0.3245181532944868</v>
       </c>
       <c r="G60" s="3">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>0.23935454952935906</v>
       </c>
       <c r="H60" s="3">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>7.3957866427610944E-2</v>
       </c>
       <c r="N60" s="2">
@@ -3568,19 +3568,19 @@
         <v>77</v>
       </c>
       <c r="E61" s="3">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>0.39856373429084385</v>
       </c>
       <c r="F61" s="3">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>0.29443447037701981</v>
       </c>
       <c r="G61" s="3">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>0.23429084380610415</v>
       </c>
       <c r="H61" s="3">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>7.2710951526032325E-2</v>
       </c>
       <c r="N61" s="2">
@@ -3596,19 +3596,19 @@
         <v>77</v>
       </c>
       <c r="E62" s="3">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>0.37345132743362836</v>
       </c>
       <c r="F62" s="3">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>0.2787610619469027</v>
       </c>
       <c r="G62" s="3">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>0.26548672566371689</v>
       </c>
       <c r="H62" s="3">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>8.2300884955752218E-2</v>
       </c>
       <c r="N62" s="2">
@@ -3624,19 +3624,19 @@
         <v>77</v>
       </c>
       <c r="E63" s="3">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>0.26530612244897955</v>
       </c>
       <c r="F63" s="3">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>0.28826530612244894</v>
       </c>
       <c r="G63" s="3">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>0.34056122448979587</v>
       </c>
       <c r="H63" s="3">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>0.10586734693877549</v>
       </c>
       <c r="N63" s="2">
@@ -3652,19 +3652,19 @@
         <v>77</v>
       </c>
       <c r="E64" s="3">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>0.38359908883826882</v>
       </c>
       <c r="F64" s="3">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>0.34988610478359911</v>
       </c>
       <c r="G64" s="3">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>0.20364464692482914</v>
       </c>
       <c r="H64" s="3">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>6.2870159453302973E-2</v>
       </c>
       <c r="N64" s="2">
@@ -3680,19 +3680,19 @@
         <v>77</v>
       </c>
       <c r="E65" s="3">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>0.37345132743362836</v>
       </c>
       <c r="F65" s="3">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>0.2787610619469027</v>
       </c>
       <c r="G65" s="3">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>0.26548672566371689</v>
       </c>
       <c r="H65" s="3">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>8.2300884955752218E-2</v>
       </c>
       <c r="N65" s="2">
@@ -3708,19 +3708,19 @@
         <v>77</v>
       </c>
       <c r="E66" s="3">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>0.35137533274179239</v>
       </c>
       <c r="F66" s="3">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>0.3105590062111801</v>
       </c>
       <c r="G66" s="3">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>0.25820763087843834</v>
       </c>
       <c r="H66" s="3">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>7.9858030168589167E-2</v>
       </c>
       <c r="N66" s="2">
@@ -3736,19 +3736,19 @@
         <v>77</v>
       </c>
       <c r="E67" s="3">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>0.37345132743362836</v>
       </c>
       <c r="F67" s="3">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>0.2787610619469027</v>
       </c>
       <c r="G67" s="3">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>0.26548672566371689</v>
       </c>
       <c r="H67" s="3">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>8.2300884955752218E-2</v>
       </c>
       <c r="N67" s="2">

</xml_diff>